<commit_message>
Job search run 2026-10-08: add top 10 new matches, mark 3 closed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GznzeDz7Dz7sjS15B4oWSX
</commit_message>
<xml_diff>
--- a/Harpreet_Job_Matches.xlsx
+++ b/Harpreet_Job_Matches.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Search Criteria" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +48,7 @@
       <color rgb="00C00000"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -145,6 +150,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -638,7 +652,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -696,7 +710,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -754,7 +768,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -812,7 +826,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -822,58 +836,58 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Thomson Reuters</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>AI &amp; Automation Engineer</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Bengaluru / Hyderabad</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>Not specified (IC role, not senior-titled)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="14" t="inlineStr">
         <is>
           <t>Redesign manual ops processes with agentic AI + automation; integrate LLMs with semantic layers, data warehouses and APIs; build RAG over structured business metadata; event-driven pipelines.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="14" t="inlineStr">
         <is>
           <t>Rare match for your metric semantic layer, text-to-SQL grounding and SQMF agentic compliance automation work.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="14" t="inlineStr">
         <is>
           <t>https://thomsonreuters.wd5.myworkdayjobs.com/External_Career_Site/job/India-Bengaluru-Karnataka/AI---Automation-Engineer_JREQ201411-1</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -928,7 +942,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -986,7 +1000,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1044,7 +1058,7 @@
       </c>
       <c r="K9" s="16" t="inlineStr">
         <is>
-          <t>❌ Closed / link not working (2026-09-30)</t>
+          <t>❌ Closed / link not working (2026-10-08)</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1102,7 +1116,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1160,7 +1174,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1218,7 +1232,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1276,7 +1290,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1334,7 +1348,7 @@
       </c>
       <c r="K14" s="16" t="inlineStr">
         <is>
-          <t>❌ Closed / link not working (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L14" s="17" t="inlineStr">
@@ -1392,7 +1406,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1402,58 +1416,58 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Applied Scientist, CMT</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>No minimum years listed (Applied Scientist I level)</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="19" t="n">
         <v>0.74</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>Competitive Monitoring team: ML, LLMs in production and recommender systems for product similarity and price recommendations.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>Production LLMs + recommendations (you built adaptive recommendation logic in APRE).</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/jobs/10530901/applied-scientist-cmt</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L16" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -1508,7 +1522,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1566,7 +1580,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1624,7 +1638,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1682,7 +1696,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -1740,7 +1754,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-09-30)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1749,8 +1763,588 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Applied AI Engineer</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Build LLM-powered applications and internal AI systems end to end; evaluate them, find where they fail and measure whether they worked; bonus for GTM/marketing data systems.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Matches your shipped LLM pipelines, evaluation/error analysis and output logging; fully remote, global hiring.</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/b8a111fa-9fd5-44d0-97ed-8fd1280be4ef</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L22" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Elastic</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Agentic AI Engineer</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Not specified (asks for deep hands-on LLM experience)</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Build self-directed multi-agent and agent-to-agent (A2A) systems for Elastic IT: LangGraph/LangChain orchestration, state management, task delegation, RAG/hybrid search, LLM observability and evals.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Near-exact match: 68-tool agent orchestration, LangGraph, RAG, LLM logging/evaluation and token-cost control.</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.elastic.co/jobs?gh_jid=8247206&amp;gh_jid=8247206</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L23" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Full-stack Engineer - Creative Agents</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Full-stack engineer on Creative Agents: UI, backend services, APIs and data models; production agents, evaluations and MCP integrations in a small fast team.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Full-stack TypeScript/React + production agents, evals and MCP are all on your resume.</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/0b3a97d4-193c-4b47-9888-7ef5803ed945</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L24" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Full-Stack Engineer (Backend Leaning) - Creative Agents</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Backend-leaning full-stack role building agent infrastructure for Creative Agents: prompts, tools, execution logic, evaluations, async workers, WebSockets.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Agent tool/execution design plus Node/Express and async pipeline experience (APRE, real-time PvP).</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/35813150-a851-4821-b732-a037b4e6c4fe</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L25" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Philips</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Full stack -  AI Application Engineer - People Analytics</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Not specified ('relevant professional experience')</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Build internal AI apps, FastAPI REST APIs, Streamlit/Dash tools, CI/CD and monitoring so People Analytics AI products reach production.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>FastAPI, CI/CD, testing and productionising AI apps; your governance platform served 2,000+ employees.</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Full-stack----AI-Application-Engineer---People-Analytics_588990-1</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L26" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Philips</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist - AI and LLMs - People Analytics</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist for People Analytics combining statistics and ML with LLM solutions: prompt workflows, semantic search, RAG and text analytics.</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Statistical modelling + RAG/semantic search + responsible AI guardrails.</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Data-Scientist---AI-and-LLMs---People-Analytics_588995-1</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L27" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>SDE II - Gen AI</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2–5 yrs</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>SDE II – Gen AI: build GenAI/computer-vision model pipelines from training to on-device deployment, optimising latency, memory and model footprint (PyTorch).</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>You shipped on-device neural inference (Maia via ONNX Runtime Web) plus PyTorch; 2-year minimum fits.</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7846609</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L28" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Applied Scientist, SSG Science</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>No minimum years (Bachelor's)</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Applied Scientist (SSG): quantize, prune, distill and fine-tune GenAI models for Amazon edge devices on the Neural Edge Engine.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>LoRA/QLoRA fine-tuning and on-device inference experience; entry-level Applied Scientist bar.</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.jobs/en/jobs/10572900/applied-scientist-ssg-science</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L29" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Applied Scientist, FinAuto</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>No minimum years listed</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Applied Scientist (FinAuto): ML, statistics and causal inference on large financial transaction data to automate and optimise finance processes.</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Financial-data ML, feature engineering and backtesting from your quant research.</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.jobs/en/jobs/10571470/applied-scientist-finauto</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L30" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Lowe's</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer_Java_ReactJS_Data&amp;ML</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2–5 yrs</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Software Engineer (Data &amp; ML): data/feature pipelines, ML/MLOps, cloud-native services and AI-enabled engineering across the SDLC (Java, React).</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Data pipelines, ML deployment and React; Java is the gap.</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>https://lowes.wd5.myworkdayjobs.com/LWS_External_CS/job/Bengaluru/Software-Engineer-Java-ReactJS-Data-ML_JR-02622143</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+        </is>
+      </c>
+      <c r="L31" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:L31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -1772,6 +2366,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1843,14 +2447,14 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1871,14 +2475,14 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1899,14 +2503,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1927,14 +2531,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>291</v>
+        <v>318</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1955,14 +2559,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -1990,7 +2594,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2622,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2039,14 +2643,14 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2067,14 +2671,14 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2095,14 +2699,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>316</v>
+        <v>275</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2123,14 +2727,14 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>636</v>
+        <v>648</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2151,14 +2755,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2790,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2207,14 +2811,14 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2235,14 +2839,14 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2263,14 +2867,14 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2291,14 +2895,14 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2319,14 +2923,14 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2958,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2375,14 +2979,14 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2403,14 +3007,14 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2431,14 +3035,14 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2466,7 +3070,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2487,14 +3091,14 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2515,14 +3119,14 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2550,7 +3154,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2571,14 +3175,14 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2599,14 +3203,14 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2634,7 +3238,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2655,14 +3259,14 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>399</v>
+        <v>424</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2683,14 +3287,14 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2711,14 +3315,14 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2739,14 +3343,14 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2767,14 +3371,14 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2802,7 +3406,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2823,14 +3427,14 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2851,14 +3455,14 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>882</v>
+        <v>894</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2879,14 +3483,14 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2907,14 +3511,14 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2935,14 +3539,14 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2963,14 +3567,14 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -2991,14 +3595,14 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3019,14 +3623,14 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3047,14 +3651,14 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3075,14 +3679,14 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3103,14 +3707,14 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>390</v>
+        <v>417</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3131,14 +3735,14 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>183</v>
+        <v>141</v>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3159,14 +3763,14 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3187,14 +3791,14 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3215,14 +3819,14 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3243,14 +3847,14 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3271,14 +3875,14 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3299,14 +3903,14 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3327,14 +3931,14 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3966,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3383,14 +3987,14 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3411,14 +4015,14 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3446,7 +4050,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3474,7 +4078,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3495,14 +4099,14 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3523,14 +4127,14 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>296</v>
+        <v>335</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3558,7 +4162,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3579,14 +4183,14 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3614,7 +4218,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3635,14 +4239,14 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3670,7 +4274,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3691,14 +4295,14 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3726,7 +4330,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3747,14 +4351,14 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E70" t="n">
         <v>0</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3782,7 +4386,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3810,7 +4414,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3831,14 +4435,14 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E73" t="n">
         <v>0</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3859,14 +4463,14 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E74" t="n">
         <v>0</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3894,7 +4498,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3915,14 +4519,14 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E76" t="n">
         <v>0</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3943,14 +4547,14 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3971,14 +4575,14 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3999,14 +4603,14 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="E79" t="n">
         <v>2</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4027,14 +4631,14 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E80" t="n">
         <v>0</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4055,14 +4659,14 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4083,14 +4687,14 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E82" t="n">
         <v>0</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4111,14 +4715,14 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E83" t="n">
         <v>0</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4139,14 +4743,14 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="E84" t="n">
         <v>0</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4167,14 +4771,14 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4806,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4223,14 +4827,14 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E87" t="n">
         <v>0</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4251,14 +4855,14 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E88" t="n">
         <v>0</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4279,14 +4883,14 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E89" t="n">
         <v>0</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4918,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4335,14 +4939,14 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>349</v>
+        <v>371</v>
       </c>
       <c r="E91" t="n">
         <v>0</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4363,14 +4967,14 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>838</v>
+        <v>815</v>
       </c>
       <c r="E92" t="n">
         <v>1</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4398,7 +5002,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4419,14 +5023,14 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E94" t="n">
         <v>0</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4447,14 +5051,14 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4475,14 +5079,14 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E96" t="n">
         <v>0</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4503,14 +5107,14 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E97" t="n">
         <v>0</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4531,14 +5135,14 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E98" t="n">
         <v>0</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4559,14 +5163,14 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E99" t="n">
         <v>0</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4587,14 +5191,14 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E100" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4615,14 +5219,14 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E101" t="n">
         <v>0</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4650,7 +5254,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4671,14 +5275,14 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>151</v>
+        <v>179</v>
       </c>
       <c r="E103" t="n">
         <v>0</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4706,7 +5310,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4727,14 +5331,14 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E105" t="n">
         <v>0</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4755,14 +5359,14 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E106" t="n">
         <v>0</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4790,7 +5394,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4811,14 +5415,14 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E108" t="n">
         <v>0</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4846,7 +5450,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4867,14 +5471,14 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E110" t="n">
         <v>0</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4895,14 +5499,14 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E111" t="n">
         <v>0</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4923,14 +5527,14 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E112" t="n">
         <v>0</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4951,14 +5555,14 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="E113" t="n">
         <v>0</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -4979,14 +5583,14 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E114" t="n">
         <v>0</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5007,14 +5611,14 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E115" t="n">
         <v>0</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5035,14 +5639,14 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E116" t="n">
         <v>0</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5063,14 +5667,14 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E117" t="n">
         <v>0</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5091,14 +5695,14 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E118" t="n">
         <v>0</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5119,14 +5723,14 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E119" t="n">
         <v>0</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5147,14 +5751,14 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E120" t="n">
         <v>0</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5175,14 +5779,14 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E121" t="n">
         <v>0</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5203,14 +5807,14 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E122" t="n">
         <v>0</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5231,14 +5835,14 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E123" t="n">
         <v>0</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5259,14 +5863,14 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="E124" t="n">
         <v>1</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5287,14 +5891,14 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E125" t="n">
         <v>0</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5315,14 +5919,14 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>692</v>
+        <v>708</v>
       </c>
       <c r="E126" t="n">
         <v>0</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5343,14 +5947,14 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E127" t="n">
         <v>0</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5378,7 +5982,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5399,14 +6003,14 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E129" t="n">
         <v>0</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5427,14 +6031,14 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E130" t="n">
         <v>0</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5455,14 +6059,14 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E131" t="n">
         <v>0</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5483,14 +6087,14 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E132" t="n">
         <v>0</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5518,7 +6122,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5539,14 +6143,14 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>710</v>
+        <v>724</v>
       </c>
       <c r="E134" t="n">
         <v>0</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5567,14 +6171,14 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E135" t="n">
         <v>0</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5595,14 +6199,14 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E136" t="n">
         <v>1</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5623,14 +6227,14 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="E137" t="n">
         <v>0</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5651,14 +6255,14 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E138" t="n">
         <v>0</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5679,14 +6283,14 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E139" t="n">
         <v>0</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5707,14 +6311,14 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E140" t="n">
         <v>0</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5735,14 +6339,14 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E141" t="n">
         <v>0</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5763,14 +6367,14 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E142" t="n">
         <v>1</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5791,14 +6395,14 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E143" t="n">
         <v>0</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5819,14 +6423,14 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E144" t="n">
         <v>0</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5847,14 +6451,14 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E145" t="n">
         <v>0</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5882,7 +6486,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5903,14 +6507,14 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E147" t="n">
         <v>0</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5931,14 +6535,14 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E148" t="n">
         <v>0</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5959,14 +6563,14 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="E149" t="n">
         <v>0</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -5987,14 +6591,14 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E150" t="n">
         <v>0</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6015,14 +6619,14 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E151" t="n">
         <v>0</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6043,14 +6647,14 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E152" t="n">
         <v>0</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6078,7 +6682,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6099,14 +6703,14 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E154" t="n">
         <v>0</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6127,14 +6731,14 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E155" t="n">
         <v>0</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6766,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6794,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -6211,14 +6815,14 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E158" t="n">
         <v>0</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Job search run 2026-10-18: add 3 new matches, mark 13 closed; skip re-posted roles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GznzeDz7Dz7sjS15B4oWSX
</commit_message>
<xml_diff>
--- a/Harpreet_Job_Matches.xlsx
+++ b/Harpreet_Job_Matches.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Search Criteria" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,6 +157,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -524,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -652,7 +655,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -710,7 +713,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -768,7 +771,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -826,7 +829,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -884,7 +887,7 @@
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>❌ Closed / link not working (2026-10-08)</t>
+          <t>❌ Closed / link not working (2026-10-18)</t>
         </is>
       </c>
       <c r="L6" s="17" t="inlineStr">
@@ -942,7 +945,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -952,58 +955,58 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Mastercard</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>AI Engineer</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Pune</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Not specified (mid-level; 'assist/support' scope)</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" s="18" t="n">
         <v>0.86</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>Develop GenAI solutions with LLMs, agentic frameworks and RAG; build AI/ML pipelines on Azure/Databricks/AWS; LLMOps, responsible AI, hallucination mitigation.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="14" t="inlineStr">
         <is>
           <t>LLM apps + RAG + guardrails + cloud deployment align with your Engineering &amp; Deployment skills.</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="14" t="inlineStr">
         <is>
           <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/AI-Engineer_R-279646</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -1058,7 +1061,7 @@
       </c>
       <c r="K9" s="16" t="inlineStr">
         <is>
-          <t>❌ Closed / link not working (2026-10-08)</t>
+          <t>❌ Closed / link not working (2026-10-18)</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1068,58 +1071,58 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Applied AI Engineer</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Bengaluru (Remote) / Delhi / Mumbai</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Hybrid/Remote</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>Not specified (stretch — customer-facing, high bar)</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="18" t="n">
         <v>0.85</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="14" t="inlineStr">
         <is>
           <t>Partner with enterprises to design, build, evaluate and launch production AI systems; write/debug code, build eval systems, handle reliability, latency, cost and safety trade-offs.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="14" t="inlineStr">
         <is>
           <t>Your cost-optimised batch LLM pipeline, evals and fallback design fit; apply as a stretch role.</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="14" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/openai/bf036b23-cd23-46d0-a02f-4b1483f4698a</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -1174,7 +1177,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1232,7 +1235,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1290,7 +1293,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1348,7 +1351,7 @@
       </c>
       <c r="K14" s="16" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L14" s="17" t="inlineStr">
@@ -1406,7 +1409,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1464,7 +1467,7 @@
       </c>
       <c r="K16" s="16" t="inlineStr">
         <is>
-          <t>❌ Closed / link not working (2026-10-08)</t>
+          <t>❌ Closed / link not working (2026-10-18)</t>
         </is>
       </c>
       <c r="L16" s="17" t="inlineStr">
@@ -1474,58 +1477,58 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Machine Learning Engineer II, EU INTech - Exports, Emerging and Expansions</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>2+ yrs professional software development</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
+      <c r="G17" s="19" t="n">
         <v>0.7</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>ML Engineer II in Amazon search (EU expansion): build ML-in-search features, analyse large data, run statistically rigorous experiments.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="14" t="inlineStr">
         <is>
           <t>Python/ML engineering + experimentation background from quant research.</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/jobs/10418966/machine-learning-engineer-ii-eu-intech-exports-emerging-and-expansions</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -1580,7 +1583,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1638,7 +1641,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1648,58 +1651,58 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Data Scientist, Alexa AI</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>2+ yrs data/research scientist</t>
         </is>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="19" t="n">
         <v>0.65</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="14" t="inlineStr">
         <is>
           <t>Data Scientist, Alexa AI: data experiments and algorithms for speech &amp; language technology (ASR, NLU).</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" s="14" t="inlineStr">
         <is>
           <t>NLP + data analysis + experimentation; SQL/Python strength.</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J20" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/jobs/10516477/data-scientist-alexa-ai</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L20" s="17" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>
@@ -1754,7 +1757,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1764,116 +1767,116 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>ElevenLabs</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Applied AI Engineer</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>Remote – Global</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>Not specified (IC role)</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="G22" s="18" t="n">
         <v>0.9</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="14" t="inlineStr">
         <is>
           <t>Build LLM-powered applications and internal AI systems end to end; evaluate them, find where they fail and measure whether they worked; bonus for GTM/marketing data systems.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I22" s="14" t="inlineStr">
         <is>
           <t>Matches your shipped LLM pipelines, evaluation/error analysis and output logging; fully remote, global hiring.</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="14" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/elevenlabs/b8a111fa-9fd5-44d0-97ed-8fd1280be4ef</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L22" s="20" t="inlineStr">
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L22" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Elastic</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Agentic AI Engineer</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Not specified (asks for deep hands-on LLM experience)</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="G23" s="18" t="n">
         <v>0.88</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="14" t="inlineStr">
         <is>
           <t>Build self-directed multi-agent and agent-to-agent (A2A) systems for Elastic IT: LangGraph/LangChain orchestration, state management, task delegation, RAG/hybrid search, LLM observability and evals.</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I23" s="14" t="inlineStr">
         <is>
           <t>Near-exact match: 68-tool agent orchestration, LangGraph, RAG, LLM logging/evaluation and token-cost control.</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J23" s="14" t="inlineStr">
         <is>
           <t>https://jobs.elastic.co/jobs?gh_jid=8247206&amp;gh_jid=8247206</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L23" s="20" t="inlineStr">
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L23" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
@@ -1928,7 +1931,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L24" s="20" t="inlineStr">
@@ -1986,7 +1989,7 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L25" s="20" t="inlineStr">
@@ -1996,116 +1999,116 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Philips</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>Full stack -  AI Application Engineer - People Analytics</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Not specified ('relevant professional experience')</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="G26" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="14" t="inlineStr">
         <is>
           <t>Build internal AI apps, FastAPI REST APIs, Streamlit/Dash tools, CI/CD and monitoring so People Analytics AI products reach production.</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="14" t="inlineStr">
         <is>
           <t>FastAPI, CI/CD, testing and productionising AI apps; your governance platform served 2,000+ employees.</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J26" s="14" t="inlineStr">
         <is>
           <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Full-stack----AI-Application-Engineer---People-Analytics_588990-1</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L26" s="20" t="inlineStr">
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L26" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>Philips</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>Data Scientist - AI and LLMs - People Analytics</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="G27" s="15" t="n">
         <v>0.78</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>Data Scientist for People Analytics combining statistics and ML with LLM solutions: prompt workflows, semantic search, RAG and text analytics.</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="14" t="inlineStr">
         <is>
           <t>Statistical modelling + RAG/semantic search + responsible AI guardrails.</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J27" s="14" t="inlineStr">
         <is>
           <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Data-Scientist---AI-and-LLMs---People-Analytics_588995-1</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L27" s="20" t="inlineStr">
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L27" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
@@ -2160,7 +2163,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L28" s="20" t="inlineStr">
@@ -2170,116 +2173,116 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Applied Scientist, SSG Science</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>No minimum years (Bachelor's)</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n">
+      <c r="G29" s="19" t="n">
         <v>0.68</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="14" t="inlineStr">
         <is>
           <t>Applied Scientist (SSG): quantize, prune, distill and fine-tune GenAI models for Amazon edge devices on the Neural Edge Engine.</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I29" s="14" t="inlineStr">
         <is>
           <t>LoRA/QLoRA fine-tuning and on-device inference experience; entry-level Applied Scientist bar.</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/jobs/10572900/applied-scientist-ssg-science</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L29" s="20" t="inlineStr">
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L29" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>Applied Scientist, FinAuto</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>No minimum years listed</t>
         </is>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G30" s="19" t="n">
         <v>0.68</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="14" t="inlineStr">
         <is>
           <t>Applied Scientist (FinAuto): ML, statistics and causal inference on large financial transaction data to automate and optimise finance processes.</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I30" s="14" t="inlineStr">
         <is>
           <t>Financial-data ML, feature engineering and backtesting from your quant research.</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J30" s="14" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/jobs/10571470/applied-scientist-finauto</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
-        </is>
-      </c>
-      <c r="L30" s="20" t="inlineStr">
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>❌ Closed / link not working (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L30" s="21" t="inlineStr">
         <is>
           <t>2026-10-08</t>
         </is>
@@ -2334,7 +2337,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-08)</t>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
       <c r="L31" s="20" t="inlineStr">
@@ -2343,8 +2346,182 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Data Scientist I</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Not specified (Data Scientist I – entry level)</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Build GenAI applications for AML transaction monitoring: RAG, Model Context Protocol (MCP), tool calling and LangChain/LangGraph workflows; LLM fine-tuning pipelines; multimodal content generation.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Near-exact match: RAG, MCP, tool calling, LangGraph, LoRA/QLoRA fine-tuning, plus your compliance-automation (SQMF) work.</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Data-Scientist-I_R-278159</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L32" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Bureau</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Associate Data Scientist</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>1–3 yrs DS/AI/ML (internships count)</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Associate Data Scientist: build features and components for graph-native models (GNNs, embeddings) for fraud/risk; take models from notebook toward production.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Python/SQL, embeddings, anomaly detection and production ML; fraud/compliance data exposure from SQMF.</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/bureau/2b7f3dda-fba7-499c-934d-b0fdfb21fe08</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L33" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Warner Bros. Discovery</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning Engineer II ( Growth &amp; ML), Hyderabad</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>2–4 yrs ML/DS (or 1–2 with relevant degree)</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>ML Engineer II on the Data &amp; Audience Platform: build and maintain production ML pipelines, probabilistic identity graphs, model development and pipeline reliability.</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Production data/ML pipelines, data-quality monitoring and feature engineering.</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>https://warnerbros.wd5.myworkdayjobs.com/global/job/Hyderabad---Phoenix-Equinox-Tower-2/Machine-Learning-Engineer-II---Data---Audience-Platform-Team---Hyderabad_R000106139</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L34" s="20" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L31"/>
+  <autoFilter ref="A1:L34"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -2376,6 +2553,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2454,7 +2634,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2475,14 +2655,14 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2503,14 +2683,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2531,14 +2711,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2559,14 +2739,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2587,14 +2767,14 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2802,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2830,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2671,14 +2851,14 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2699,14 +2879,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="E11" t="n">
         <v>8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2727,14 +2907,14 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2755,14 +2935,14 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2783,14 +2963,14 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2811,14 +2991,14 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2839,14 +3019,14 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2867,14 +3047,14 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2895,14 +3075,14 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2923,14 +3103,14 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2958,7 +3138,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2979,14 +3159,14 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3007,14 +3187,14 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3035,14 +3215,14 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3250,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3091,14 +3271,14 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3119,14 +3299,14 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3147,14 +3327,14 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3175,14 +3355,14 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3203,14 +3383,14 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3418,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3259,14 +3439,14 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3287,14 +3467,14 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3315,14 +3495,14 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3343,14 +3523,14 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3371,14 +3551,14 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3399,14 +3579,14 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3614,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3455,14 +3635,14 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3483,14 +3663,14 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3511,14 +3691,14 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3539,14 +3719,14 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3754,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3595,14 +3775,14 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3623,14 +3803,14 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3651,14 +3831,14 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3679,14 +3859,14 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3707,14 +3887,14 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>417</v>
+        <v>380</v>
       </c>
       <c r="E47" t="n">
         <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3735,14 +3915,14 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="E48" t="n">
         <v>3</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3763,14 +3943,14 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3791,14 +3971,14 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E50" t="n">
         <v>0</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3819,14 +3999,14 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E51" t="n">
         <v>0</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3847,14 +4027,14 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3875,14 +4055,14 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E53" t="n">
         <v>0</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3903,14 +4083,14 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3931,14 +4111,14 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E55" t="n">
         <v>0</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3959,14 +4139,14 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3987,14 +4167,14 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="E57" t="n">
         <v>1</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4015,14 +4195,14 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E58" t="n">
         <v>1</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4043,14 +4223,14 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59" t="n">
         <v>0</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4071,14 +4251,14 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4099,14 +4279,14 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4127,14 +4307,14 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4155,14 +4335,14 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E63" t="n">
         <v>1</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4183,14 +4363,14 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4398,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4239,14 +4419,14 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4454,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4295,14 +4475,14 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4510,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4538,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4379,14 +4559,14 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E71" t="n">
         <v>0</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4594,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4435,14 +4615,14 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E73" t="n">
         <v>0</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4463,14 +4643,14 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E74" t="n">
         <v>0</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4491,14 +4671,14 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4519,14 +4699,14 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E76" t="n">
         <v>0</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4547,14 +4727,14 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4575,14 +4755,14 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4603,14 +4783,14 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4631,14 +4811,14 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E80" t="n">
         <v>0</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4659,14 +4839,14 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4874,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4715,14 +4895,14 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E83" t="n">
         <v>0</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4743,14 +4923,14 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>392</v>
+        <v>401</v>
       </c>
       <c r="E84" t="n">
         <v>0</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4771,14 +4951,14 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4986,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4827,14 +5007,14 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E87" t="n">
         <v>0</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4855,14 +5035,14 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E88" t="n">
         <v>0</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4883,14 +5063,14 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E89" t="n">
         <v>0</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4911,14 +5091,14 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E90" t="n">
         <v>1</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4939,14 +5119,14 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>371</v>
+        <v>393</v>
       </c>
       <c r="E91" t="n">
         <v>0</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4967,14 +5147,14 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="E92" t="n">
         <v>1</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4995,14 +5175,14 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E93" t="n">
         <v>0</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5023,14 +5203,14 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E94" t="n">
         <v>0</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5051,14 +5231,14 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5079,14 +5259,14 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E96" t="n">
         <v>0</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5107,14 +5287,14 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="E97" t="n">
         <v>0</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5135,14 +5315,14 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E98" t="n">
         <v>0</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5163,14 +5343,14 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E99" t="n">
         <v>0</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5191,14 +5371,14 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E100" t="n">
         <v>2</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5406,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5254,7 +5434,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5275,14 +5455,14 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="E103" t="n">
         <v>0</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5303,14 +5483,14 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="E104" t="n">
         <v>0</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5338,7 +5518,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5546,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5574,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5602,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5630,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5471,14 +5651,14 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E110" t="n">
         <v>0</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5499,14 +5679,14 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E111" t="n">
         <v>0</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5527,14 +5707,14 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E112" t="n">
         <v>0</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5555,14 +5735,14 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="E113" t="n">
         <v>0</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5583,14 +5763,14 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E114" t="n">
         <v>0</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5611,14 +5791,14 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E115" t="n">
         <v>0</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5639,14 +5819,14 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E116" t="n">
         <v>0</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5667,14 +5847,14 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="E117" t="n">
         <v>0</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5695,14 +5875,14 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E118" t="n">
         <v>0</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5723,14 +5903,14 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="E119" t="n">
         <v>0</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5758,7 +5938,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5779,14 +5959,14 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E121" t="n">
         <v>0</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5807,14 +5987,14 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>240</v>
+        <v>262</v>
       </c>
       <c r="E122" t="n">
         <v>0</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5835,14 +6015,14 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="E123" t="n">
         <v>0</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5863,14 +6043,14 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E124" t="n">
         <v>1</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5891,14 +6071,14 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E125" t="n">
         <v>0</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5919,14 +6099,14 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="E126" t="n">
         <v>0</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5947,14 +6127,14 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="E127" t="n">
         <v>0</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5975,14 +6155,14 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E128" t="n">
         <v>0</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6010,7 +6190,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6031,14 +6211,14 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E130" t="n">
         <v>0</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6066,7 +6246,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6087,14 +6267,14 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E132" t="n">
         <v>0</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6115,14 +6295,14 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E133" t="n">
         <v>0</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6143,14 +6323,14 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>724</v>
+        <v>731</v>
       </c>
       <c r="E134" t="n">
         <v>0</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6178,7 +6358,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6199,14 +6379,14 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E136" t="n">
         <v>1</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6227,14 +6407,14 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="E137" t="n">
         <v>0</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6255,14 +6435,14 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E138" t="n">
         <v>0</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6283,14 +6463,14 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E139" t="n">
         <v>0</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6311,14 +6491,14 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E140" t="n">
         <v>0</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6339,14 +6519,14 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E141" t="n">
         <v>0</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6367,14 +6547,14 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E142" t="n">
         <v>1</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6395,14 +6575,14 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E143" t="n">
         <v>0</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6610,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6458,7 +6638,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6486,7 +6666,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6507,14 +6687,14 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E147" t="n">
         <v>0</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6535,14 +6715,14 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E148" t="n">
         <v>0</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6563,14 +6743,14 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>310</v>
+        <v>319</v>
       </c>
       <c r="E149" t="n">
         <v>0</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6591,14 +6771,14 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E150" t="n">
         <v>0</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6619,14 +6799,14 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6834,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6862,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6703,14 +6883,14 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E154" t="n">
         <v>0</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6731,14 +6911,14 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E155" t="n">
         <v>0</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6946,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6794,7 +6974,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6815,14 +6995,14 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E158" t="n">
         <v>0</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restart job tracker for updated resume, focused on AI Engineer / FDE roles
Reset seen_jobs and the spreadsheet, refresh profile.md, keep DS/ML titles
only when the work is clearly LLM/agent focused, and let update_sheet.py
create a new workbook when none exists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GznzeDz7Dz7sjS15B4oWSX
</commit_message>
<xml_diff>
--- a/Harpreet_Job_Matches.xlsx
+++ b/Harpreet_Job_Matches.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Search Criteria" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matching Jobs'!$A$1:$L$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,18 +34,11 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
-    </font>
-    <font>
       <b val="1"/>
     </font>
     <font>
-      <strike val="1"/>
-      <color rgb="00999999"/>
-    </font>
-    <font>
-      <color rgb="00C00000"/>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="7">
@@ -67,17 +60,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -107,10 +100,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -118,50 +117,22 @@
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -540,7 +511,7 @@
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -600,1928 +571,768 @@
           <t>Link Check (last run)</t>
         </is>
       </c>
-      <c r="L1" s="13" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date Added</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>100ms</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>AI Engineer – AI Agents (Healthcare)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>2–5 yrs SWE incl. 1–2 yrs on LLM/AI products</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Build agentic workflows for healthcare AI agents; run systematic LLM evals, track regressions, define metrics (correctness, latency, hallucination, safety); tune prompts, retrieval and fine-tuning datasets; build eval/monitoring pipelines.</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Direct match: you built a 68-tool production agent, LLM output logging, error-analysis taxonomy &amp; multi-provider fallbacks.</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Build agentic workflows for healthcare AI agents; run systematic LLM evaluations and regression tracking; define correctness/latency/hallucination/safety metrics; tune prompts, retrieval and fine-tuning datasets.</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Your 68-tool production agent, LLM output logging, error-analysis taxonomy and fallback chains map one-to-one.</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/100ms/4c9f19c7-4432-4394-ba93-167319c68adc</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Observe.AI</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>AI Agent Engineer</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>1–5 yrs (conversational AI / solutions / integrations)</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="5" t="n">
         <v>0.93</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Own end-to-end delivery of customer-facing AI agents: prompt design, workflow configuration, API/telephony integrations, evaluation frameworks, demos and deployment.</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Agent building + tool calling + evaluation + customer-facing delivery mirrors your Chessy agent and Protimart assistant.</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Forward-deployed style: own customer AI-agent delivery end to end – prompt design, workflow configuration, API/telephony integrations, evaluation frameworks, demos and deployment.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Agent building + tool calling + evals + client delivery (Developer Insights, metric governance).</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>https://www.observe.ai/position?gh_jid=5432596008</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Data Scientist I</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Not specified (Data Scientist I – entry level)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>GenAI for anti-money-laundering transaction monitoring: RAG, Model Context Protocol (MCP), tool calling, LangChain/LangGraph workflows, LLM fine-tuning pipelines.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>RAG, MCP, tool calling, LangGraph and LoRA/QLoRA are all on your resume; title is DS but the work is AI engineering.</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Data-Scientist-I_R-278159</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Cursor</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer - India</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / New Delhi / Mumbai</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not specified (stretch)</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer: discover customer bottlenecks, design and ship Cursor-powered workflows (refactors, PR review loops, incident→fix), own tracing, evals, model debugging; Python + TypeScript.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Exactly the FDE profile: client-facing agentic systems with verification checks, Python + TypeScript, tech-lead ownership.</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/cursor/166c3951-1d2a-4e61-b79b-bedefe96073b</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>AI Platform Engineer</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Build the execution layer for Supabase's internal AI OS: event-triggered queues, model-agnostic agent runtime, durable state, human review gates, logging.</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Propose/confirm human-in-the-loop gating, LLM logging and fallback chains; you build on Postgres/Supabase.</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/supabase/3b5d54ca-741b-45ac-bd3f-31605a0d3541</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Coinbase</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Machine Learning Engineer</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Remote – India</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>2+ yrs ML / software engineering</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Build the orchestration layer coordinating vendor AI, internal multi-agent systems and humans: state transitions, context sharing, intent routing across LLM frameworks; production Python services.</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Intent classification/routing, human-in-the-loop handoffs and multi-provider LLM orchestration are core to your resume.</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="G7" s="5" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Build the orchestration layer between vendor AI, internal multi-agent systems and human agents: state transitions, context sharing, intent routing across LLM frameworks; production Python services.</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Intent routing (200-intent taxonomy), human handoffs and multi-provider LLM orchestration.</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>https://www.coinbase.com/careers/positions/7985187?gh_jid=7985187</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>GitLab</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>AI Engineer</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Remote (Bangalore)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Full-Stack Engineer (Backend Leaning) - Creative Agents</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (IC role, not senior-titled)</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Embed AI into internal workflows end-to-end: discovery, prompt engineering, agent design with human-in-the-loop, guardrails, eval frameworks, integrations (REST/GraphQL, Workato, Glean).</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Asks for exactly your stack: HITL agents, guardrails, evals, Anthropic/OpenAI models, n8n-style orchestration.</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/gitlab/jobs/8556658002</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Backend-leaning full-stack engineer for Creative Agents: agent infrastructure, prompts, tools, execution logic, evaluations, async workers and WebSockets.</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Agent tool/execution design, Node/Express services and real-time systems (PvP multiplayer).</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/35813150-a851-4821-b732-a037b4e6c4fe</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Thomson Reuters</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>AI &amp; Automation Engineer</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru / Hyderabad</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Full-Stack Engineer - Creative Agents</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Remote – Global</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Not specified (IC role)</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Full-stack engineer for Creative Agents: UI, backend services, APIs and data models; production agents, evaluations and MCP integrations.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>React + TypeScript + production agents, evals and MCP.</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/elevenlabs/0b3a97d4-193c-4b47-9888-7ef5803ed945</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Bolna (YC F25)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>AI Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / Delhi</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Onsite</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Early-career</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>AI Solutions Engineer: design and iterate system prompts and tools for voice agents, build agent flows with enterprise customers, test conversations and fix failures.</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Customer-facing agent building (forward-deployed style); you may be over-qualified – good fallback.</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/bolna/131e206f-3fd9-4905-9f4c-c3fdc4c32cc9</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Bristol Myers Squibb</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer - Quality system</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>Not specified (IC role, not senior-titled)</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>Redesign manual ops processes with agentic AI + automation; integrate LLMs with semantic layers, data warehouses and APIs; build RAG over structured business metadata; event-driven pipelines.</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>Rare match for your metric semantic layer, text-to-SQL grounding and SQMF agentic compliance automation work.</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="inlineStr">
-        <is>
-          <t>https://thomsonreuters.wd5.myworkdayjobs.com/External_Career_Site/job/India-Bengaluru-Karnataka/AI---Automation-Engineer_JREQ201411-1</t>
-        </is>
-      </c>
-      <c r="K6" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L6" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>AI Platform Engineer</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Remote – Global</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (IC role)</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Build the execution layer for Supabase's internal AI OS: event-triggered queues, model-agnostic agent runtime, durable state, human review gates, logging.</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>HITL approval gates, audit trails, idempotent work items — plus you already build on Supabase/Postgres.</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/supabase/3b5d54ca-741b-45ac-bd3f-31605a0d3541</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Minimum 2 yrs (early-career)</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>AI Engineer for pharma Quality: build AI-enabled solutions with Quality stakeholders, data prep/validation for AI models, LIMS integration, testing and deployment in a compliant environment.</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Stakeholder-facing AI delivery with verification and audit discipline.</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>https://bristolmyerssquibb.wd5.myworkdayjobs.com/BMS/job/Hyderabad---TS---IN/Quality-system-analyst_R1605789</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>AI Engineer</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="inlineStr">
-        <is>
-          <t>Not specified (mid-level; 'assist/support' scope)</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>Develop GenAI solutions with LLMs, agentic frameworks and RAG; build AI/ML pipelines on Azure/Databricks/AWS; LLMOps, responsible AI, hallucination mitigation.</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>LLM apps + RAG + guardrails + cloud deployment align with your Engineering &amp; Deployment skills.</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="inlineStr">
-        <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/AI-Engineer_R-279646</t>
-        </is>
-      </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L8" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>AI Engineer</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Gurugram</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Design, build and deploy LLM, agentic AI and RAG solutions for pricing/interchange strategy; vector embeddings, semantic search, Python APIs/microservices.</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>Agentic AI, RAG, embeddings and semantic search in production — all on your resume.</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="inlineStr">
-        <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Gurgaon-India/AI-Engineer_R-291884</t>
-        </is>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Applied AI Engineer</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru (Remote) / Delhi / Mumbai</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid/Remote</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>Not specified (stretch — customer-facing, high bar)</t>
-        </is>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Partner with enterprises to design, build, evaluate and launch production AI systems; write/debug code, build eval systems, handle reliability, latency, cost and safety trade-offs.</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>Your cost-optimised batch LLM pipeline, evals and fallback design fit; apply as a stretch role.</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/openai/bf036b23-cd23-46d0-a02f-4b1483f4698a</t>
-        </is>
-      </c>
-      <c r="K10" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L10" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Cursor</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineer - India</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru / New Delhi / Mumbai</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Glance</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>SDE II - Gen AI</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (stretch)</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Forward Deployed Engineer: design and ship Cursor-powered workflows for enterprise customers (refactors, PR review loops), own tracing/evals/model debugging; Python + TypeScript.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>End-to-end AI builder with Python + TypeScript and production LLM debugging; strong tech-lead signal.</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/cursor/166c3951-1d2a-4e61-b79b-bedefe96073b</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>2–5 yrs</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>SDE II – Gen AI: GenAI/computer-vision pipelines from training to on-device deployment, optimising latency, memory and model size (PyTorch).</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>On-device inference (Maia via ONNX Runtime Web) + PyTorch; more ML-heavy than your target.</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/glance/jobs/7846609</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Bolna (YC F25)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>AI Solutions Engineer</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru / Delhi</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Applied Scientist, Alexa International Tech</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Early-career</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Design and iterate system prompts and tools for voice AI agents, build agent flows with customers, test conversations and fix failures.</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Prompt/context engineering and tool calling for agents; fast-growing Voice-AI startup.</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/bolna/131e206f-3fd9-4905-9f4c-c3fdc4c32cc9</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Bachelor's + 2 yrs relevant experience</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Applied Scientist, Alexa International: LLM algorithms and applied AI for multilingual Alexa+ across text, speech and vision.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>LLM work fits, but it's a scientist-track role – lower priority for your AI-engineer focus.</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>https://www.amazon.jobs/en/jobs/10490052/applied-scientist-alexa-international-tech</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Sarvam AI</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Embedded Data Scientist, Chanakya</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Hevo Data</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Onsite</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>2–5 yrs data science / applied ML</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Embedded with client deployments to structure multimodal data so AI systems can reason over it: document segmentation, metadata, entities/relationships, semantic structures.</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Your machine-readable metric contract schema and lineage work maps directly to designing semantic structures for AI.</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/sarvam/dc047f4f-97be-4bb3-a9f1-cebbfc4de3e6</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2–4 yrs data engineering</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Customer-facing Solutions Engineer: be the sole technical person with Heads of Data/CTOs, design data architectures, pipelines and warehouses.</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Forward-deployed style client work + BigQuery/SQL; not AI-focused.</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/hevodata/ee02ca24-94ec-415b-ab36-7dec4d62099b</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Bristol Myers Squibb</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>AI Engineer - Quality system</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>Minimum 2 yrs</t>
-        </is>
-      </c>
-      <c r="G14" s="15" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>Develop AI-enabled solutions for pharma Quality processes; data prep/validation for AI/ML models, LIMS integration, testing &amp; deployment in a compliant environment.</t>
-        </is>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>Compliance automation, audit trails and data-quality checks (SQMF) are directly transferable.</t>
-        </is>
-      </c>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>https://bristolmyerssquibb.wd5.myworkdayjobs.com/BMS/job/Hyderabad---TS---IN/Quality-system-analyst_R1605789</t>
-        </is>
-      </c>
-      <c r="K14" s="16" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L14" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Applied Scientist, Alexa International Tech</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Bachelor's + 2 yrs relevant experience</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Applied Scientist on Alexa International: develop LLM algorithms and applied AI for multilingual Alexa+ across text, speech and vision.</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>LLM integration, NLP and fine-tuning (LoRA/QLoRA) skills; entry-level Applied Scientist bar.</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10490052/applied-scientist-alexa-international-tech</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>Applied Scientist, CMT</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>No minimum years listed (Applied Scientist I level)</t>
-        </is>
-      </c>
-      <c r="G16" s="19" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="H16" s="14" t="inlineStr">
-        <is>
-          <t>Competitive Monitoring team: ML, LLMs in production and recommender systems for product similarity and price recommendations.</t>
-        </is>
-      </c>
-      <c r="I16" s="14" t="inlineStr">
-        <is>
-          <t>Production LLMs + recommendations (you built adaptive recommendation logic in APRE).</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10530901/applied-scientist-cmt</t>
-        </is>
-      </c>
-      <c r="K16" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L16" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>Machine Learning Engineer II, EU INTech - Exports, Emerging and Expansions</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F17" s="14" t="inlineStr">
-        <is>
-          <t>2+ yrs professional software development</t>
-        </is>
-      </c>
-      <c r="G17" s="19" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>ML Engineer II in Amazon search (EU expansion): build ML-in-search features, analyse large data, run statistically rigorous experiments.</t>
-        </is>
-      </c>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>Python/ML engineering + experimentation background from quant research.</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10418966/machine-learning-engineer-ii-eu-intech-exports-emerging-and-expansions</t>
-        </is>
-      </c>
-      <c r="K17" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L17" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Applied Scientist, International Machine Learning</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>No minimum years listed</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>International Machine Learning team: design, build and deploy scalable ML models to automate and optimise India consumer businesses.</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Feature engineering, statistical modelling and ML pipelines from your trading/ML research.</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10458636/applied-scientist-international-machine-learning</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Applied Scientist I, Amazon Shipping</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Gurugram</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>No minimum years listed (Applied Scientist I)</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Forecasting &amp; optimisation for Amazon Shipping using tree models, deep learning (LSTMs, transformers), LLMs and RL.</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Time-series/financial modelling and backtesting experience transfers to forecasting.</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10557374/applied-scientist-i-amazon-shipping</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
-        <is>
-          <t>Data Scientist, Alexa AI</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F20" s="14" t="inlineStr">
-        <is>
-          <t>2+ yrs data/research scientist</t>
-        </is>
-      </c>
-      <c r="G20" s="19" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="H20" s="14" t="inlineStr">
-        <is>
-          <t>Data Scientist, Alexa AI: data experiments and algorithms for speech &amp; language technology (ASR, NLU).</t>
-        </is>
-      </c>
-      <c r="I20" s="14" t="inlineStr">
-        <is>
-          <t>NLP + data analysis + experimentation; SQL/Python strength.</t>
-        </is>
-      </c>
-      <c r="J20" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10516477/data-scientist-alexa-ai</t>
-        </is>
-      </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L20" s="17" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Hevo Data</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Solutions Engineer</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>2–4 yrs data engineering</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Customer-facing Solutions Engineer: design data architectures with Heads of Data/CTOs, pipelines, cloud warehouses.</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>dbt, BigQuery, pipelines &amp; data-quality monitoring plus tech-lead communication.</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/hevodata/ee02ca24-94ec-415b-ab36-7dec4d62099b</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>ElevenLabs</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
-        <is>
-          <t>Applied AI Engineer</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Remote – Global</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Not specified (IC role)</t>
-        </is>
-      </c>
-      <c r="G22" s="18" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
-        <is>
-          <t>Build LLM-powered applications and internal AI systems end to end; evaluate them, find where they fail and measure whether they worked; bonus for GTM/marketing data systems.</t>
-        </is>
-      </c>
-      <c r="I22" s="14" t="inlineStr">
-        <is>
-          <t>Matches your shipped LLM pipelines, evaluation/error analysis and output logging; fully remote, global hiring.</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/elevenlabs/b8a111fa-9fd5-44d0-97ed-8fd1280be4ef</t>
-        </is>
-      </c>
-      <c r="K22" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L22" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>Elastic</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>Agentic AI Engineer</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Not specified (asks for deep hands-on LLM experience)</t>
-        </is>
-      </c>
-      <c r="G23" s="18" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>Build self-directed multi-agent and agent-to-agent (A2A) systems for Elastic IT: LangGraph/LangChain orchestration, state management, task delegation, RAG/hybrid search, LLM observability and evals.</t>
-        </is>
-      </c>
-      <c r="I23" s="14" t="inlineStr">
-        <is>
-          <t>Near-exact match: 68-tool agent orchestration, LangGraph, RAG, LLM logging/evaluation and token-cost control.</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="inlineStr">
-        <is>
-          <t>https://jobs.elastic.co/jobs?gh_jid=8247206&amp;gh_jid=8247206</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L23" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>ElevenLabs</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Full-stack Engineer - Creative Agents</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Remote – Global</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (IC role)</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Full-stack engineer on Creative Agents: UI, backend services, APIs and data models; production agents, evaluations and MCP integrations in a small fast team.</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Full-stack TypeScript/React + production agents, evals and MCP are all on your resume.</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/elevenlabs/0b3a97d4-193c-4b47-9888-7ef5803ed945</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L24" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>ElevenLabs</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Full-Stack Engineer (Backend Leaning) - Creative Agents</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Remote – Global</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (IC role)</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Backend-leaning full-stack role building agent infrastructure for Creative Agents: prompts, tools, execution logic, evaluations, async workers, WebSockets.</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>Agent tool/execution design plus Node/Express and async pipeline experience (APRE, real-time PvP).</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/elevenlabs/35813150-a851-4821-b732-a037b4e6c4fe</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L25" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>Philips</t>
-        </is>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
-        <is>
-          <t>Full stack -  AI Application Engineer - People Analytics</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>Not specified ('relevant professional experience')</t>
-        </is>
-      </c>
-      <c r="G26" s="15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H26" s="14" t="inlineStr">
-        <is>
-          <t>Build internal AI apps, FastAPI REST APIs, Streamlit/Dash tools, CI/CD and monitoring so People Analytics AI products reach production.</t>
-        </is>
-      </c>
-      <c r="I26" s="14" t="inlineStr">
-        <is>
-          <t>FastAPI, CI/CD, testing and productionising AI apps; your governance platform served 2,000+ employees.</t>
-        </is>
-      </c>
-      <c r="J26" s="14" t="inlineStr">
-        <is>
-          <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Full-stack----AI-Application-Engineer---People-Analytics_588990-1</t>
-        </is>
-      </c>
-      <c r="K26" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L26" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>Philips</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>Data Scientist - AI and LLMs - People Analytics</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>Data Scientist for People Analytics combining statistics and ML with LLM solutions: prompt workflows, semantic search, RAG and text analytics.</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="inlineStr">
-        <is>
-          <t>Statistical modelling + RAG/semantic search + responsible AI guardrails.</t>
-        </is>
-      </c>
-      <c r="J27" s="14" t="inlineStr">
-        <is>
-          <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers/job/Bangalore/Data-Scientist---AI-and-LLMs---People-Analytics_588995-1</t>
-        </is>
-      </c>
-      <c r="K27" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L27" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Glance</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>SDE II - Gen AI</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>2–5 yrs</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>SDE II – Gen AI: build GenAI/computer-vision model pipelines from training to on-device deployment, optimising latency, memory and model footprint (PyTorch).</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>You shipped on-device neural inference (Maia via ONNX Runtime Web) plus PyTorch; 2-year minimum fits.</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/glance/jobs/7846609</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L28" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
-        <is>
-          <t>Applied Scientist, SSG Science</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F29" s="14" t="inlineStr">
-        <is>
-          <t>No minimum years (Bachelor's)</t>
-        </is>
-      </c>
-      <c r="G29" s="19" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H29" s="14" t="inlineStr">
-        <is>
-          <t>Applied Scientist (SSG): quantize, prune, distill and fine-tune GenAI models for Amazon edge devices on the Neural Edge Engine.</t>
-        </is>
-      </c>
-      <c r="I29" s="14" t="inlineStr">
-        <is>
-          <t>LoRA/QLoRA fine-tuning and on-device inference experience; entry-level Applied Scientist bar.</t>
-        </is>
-      </c>
-      <c r="J29" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10572900/applied-scientist-ssg-science</t>
-        </is>
-      </c>
-      <c r="K29" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L29" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="14" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>Applied Scientist, FinAuto</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>No minimum years listed</t>
-        </is>
-      </c>
-      <c r="G30" s="19" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H30" s="14" t="inlineStr">
-        <is>
-          <t>Applied Scientist (FinAuto): ML, statistics and causal inference on large financial transaction data to automate and optimise finance processes.</t>
-        </is>
-      </c>
-      <c r="I30" s="14" t="inlineStr">
-        <is>
-          <t>Financial-data ML, feature engineering and backtesting from your quant research.</t>
-        </is>
-      </c>
-      <c r="J30" s="14" t="inlineStr">
-        <is>
-          <t>https://www.amazon.jobs/en/jobs/10571470/applied-scientist-finauto</t>
-        </is>
-      </c>
-      <c r="K30" s="16" t="inlineStr">
-        <is>
-          <t>❌ Closed / link not working (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L30" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Lowe's</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer_Java_ReactJS_Data&amp;ML</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>2–5 yrs</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Software Engineer (Data &amp; ML): data/feature pipelines, ML/MLOps, cloud-native services and AI-enabled engineering across the SDLC (Java, React).</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Data pipelines, ML deployment and React; Java is the gap.</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>https://lowes.wd5.myworkdayjobs.com/LWS_External_CS/job/Bengaluru/Software-Engineer-Java-ReactJS-Data-ML_JR-02622143</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L31" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Mastercard</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Data Scientist I</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Not specified (Data Scientist I – entry level)</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Build GenAI applications for AML transaction monitoring: RAG, Model Context Protocol (MCP), tool calling and LangChain/LangGraph workflows; LLM fine-tuning pipelines; multimodal content generation.</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Near-exact match: RAG, MCP, tool calling, LangGraph, LoRA/QLoRA fine-tuning, plus your compliance-automation (SQMF) work.</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers/job/Pune-India/Data-Scientist-I_R-278159</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L32" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Bureau</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Associate Data Scientist</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Onsite</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>1–3 yrs DS/AI/ML (internships count)</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Associate Data Scientist: build features and components for graph-native models (GNNs, embeddings) for fraud/risk; take models from notebook toward production.</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Python/SQL, embeddings, anomaly detection and production ML; fraud/compliance data exposure from SQMF.</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/bureau/2b7f3dda-fba7-499c-934d-b0fdfb21fe08</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L33" s="20" t="inlineStr">
-        <is>
-          <t>2026-10-18</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Warner Bros. Discovery</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Machine Learning Engineer II ( Growth &amp; ML), Hyderabad</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Hybrid</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>2–4 yrs ML/DS (or 1–2 with relevant degree)</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>ML Engineer II on the Data &amp; Audience Platform: build and maintain production ML pipelines, probabilistic identity graphs, model development and pipeline reliability.</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Production data/ML pipelines, data-quality monitoring and feature engineering.</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>https://warnerbros.wd5.myworkdayjobs.com/global/job/Hyderabad---Phoenix-Equinox-Tower-2/Machine-Learning-Engineer-II---Data---Audience-Platform-Team---Hyderabad_R000106139</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>✅ Working – HTTP 200, posting live (2026-10-18)</t>
-        </is>
-      </c>
-      <c r="L34" s="20" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L34"/>
+  <autoFilter ref="A1:L14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -2536,26 +1347,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2579,32 +1370,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Company (board)</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Official Careers Page</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>Openings Scanned (last run)</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Jobs in Sheet</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Last Run</t>
         </is>
@@ -2616,7 +1407,7 @@
           <t>100ms</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/100ms</t>
         </is>
@@ -2644,7 +1435,7 @@
           <t>adobe</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>https://adobe.wd5.myworkdayjobs.com/external_experienced</t>
         </is>
@@ -2672,7 +1463,7 @@
           <t>affirm</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/affirm</t>
         </is>
@@ -2700,7 +1491,7 @@
           <t>agoda</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/agoda</t>
         </is>
@@ -2728,7 +1519,7 @@
           <t>airbnb</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/airbnb</t>
         </is>
@@ -2756,7 +1547,7 @@
           <t>airbyte</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/airbyte</t>
         </is>
@@ -2784,7 +1575,7 @@
           <t>airtable</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/airtable</t>
         </is>
@@ -2812,7 +1603,7 @@
           <t>alchemy</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/alchemy</t>
         </is>
@@ -2840,7 +1631,7 @@
           <t>amat</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>https://amat.wd1.myworkdayjobs.com/External</t>
         </is>
@@ -2868,7 +1659,7 @@
           <t>amazon</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>https://www.amazon.jobs/en/search?base_query=machine+learning&amp;loc_query=India</t>
         </is>
@@ -2882,7 +1673,7 @@
         <v>265</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -2896,7 +1687,7 @@
           <t>anthropic</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/anthropic</t>
         </is>
@@ -2924,7 +1715,7 @@
           <t>asana</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/asana</t>
         </is>
@@ -2952,7 +1743,7 @@
           <t>athenahealth</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>https://athenahealth.wd1.myworkdayjobs.com/External</t>
         </is>
@@ -2980,7 +1771,7 @@
           <t>atlan</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/atlan</t>
         </is>
@@ -3008,7 +1799,7 @@
           <t>attio</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/attio</t>
         </is>
@@ -3036,7 +1827,7 @@
           <t>autodesk</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>https://autodesk.wd1.myworkdayjobs.com/Ext</t>
         </is>
@@ -3064,7 +1855,7 @@
           <t>baseten</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/baseten</t>
         </is>
@@ -3092,7 +1883,7 @@
           <t>boeing</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>https://boeing.wd1.myworkdayjobs.com/EXTERNAL_CAREERS</t>
         </is>
@@ -3120,7 +1911,7 @@
           <t>bolna</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/bolna</t>
         </is>
@@ -3148,7 +1939,7 @@
           <t>brex</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/brex</t>
         </is>
@@ -3176,7 +1967,7 @@
           <t>bristolmyerssquibb</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>https://bristolmyerssquibb.wd5.myworkdayjobs.com/BMS</t>
         </is>
@@ -3204,7 +1995,7 @@
           <t>broadridge</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>https://broadridge.wd5.myworkdayjobs.com/Careers</t>
         </is>
@@ -3232,7 +2023,7 @@
           <t>browserbase</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/browserbase</t>
         </is>
@@ -3260,7 +2051,7 @@
           <t>bureau</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/bureau</t>
         </is>
@@ -3274,7 +2065,7 @@
         <v>19</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -3288,7 +2079,7 @@
           <t>capitalone</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>https://capitalone.wd12.myworkdayjobs.com/Capital_One</t>
         </is>
@@ -3316,7 +2107,7 @@
           <t>cartesia</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/cartesia</t>
         </is>
@@ -3344,7 +2135,7 @@
           <t>chime</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/chime</t>
         </is>
@@ -3372,7 +2163,7 @@
           <t>cisco</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>https://cisco.wd5.myworkdayjobs.com/Cisco_Careers</t>
         </is>
@@ -3400,7 +2191,7 @@
           <t>clerk</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/clerk</t>
         </is>
@@ -3428,7 +2219,7 @@
           <t>cloudflare</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/cloudflare</t>
         </is>
@@ -3456,7 +2247,7 @@
           <t>cognition</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/cognition</t>
         </is>
@@ -3484,7 +2275,7 @@
           <t>cohere</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/cohere</t>
         </is>
@@ -3512,7 +2303,7 @@
           <t>coinbase</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/coinbase</t>
         </is>
@@ -3540,7 +2331,7 @@
           <t>composio</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/composio</t>
         </is>
@@ -3568,7 +2359,7 @@
           <t>cred</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/cred</t>
         </is>
@@ -3596,7 +2387,7 @@
           <t>cursor</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/cursor</t>
         </is>
@@ -3624,7 +2415,7 @@
           <t>databricks</t>
         </is>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/databricks</t>
         </is>
@@ -3652,7 +2443,7 @@
           <t>datadog</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/datadog</t>
         </is>
@@ -3680,7 +2471,7 @@
           <t>decagon</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/decagon</t>
         </is>
@@ -3708,7 +2499,7 @@
           <t>deepgram</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/deepgram</t>
         </is>
@@ -3736,7 +2527,7 @@
           <t>discord</t>
         </is>
       </c>
-      <c r="B42" s="10" t="inlineStr">
+      <c r="B42" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/discord</t>
         </is>
@@ -3764,7 +2555,7 @@
           <t>dropbox</t>
         </is>
       </c>
-      <c r="B43" s="10" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/dropbox</t>
         </is>
@@ -3792,7 +2583,7 @@
           <t>druva</t>
         </is>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/druva</t>
         </is>
@@ -3820,7 +2611,7 @@
           <t>dust</t>
         </is>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/dust</t>
         </is>
@@ -3848,7 +2639,7 @@
           <t>e2b</t>
         </is>
       </c>
-      <c r="B46" s="10" t="inlineStr">
+      <c r="B46" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/e2b</t>
         </is>
@@ -3876,7 +2667,7 @@
           <t>elastic</t>
         </is>
       </c>
-      <c r="B47" s="10" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/elastic</t>
         </is>
@@ -3890,7 +2681,7 @@
         <v>380</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -3904,7 +2695,7 @@
           <t>elevenlabs</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/elevenlabs</t>
         </is>
@@ -3918,7 +2709,7 @@
         <v>156</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -3932,7 +2723,7 @@
           <t>ema</t>
         </is>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/ema</t>
         </is>
@@ -3960,7 +2751,7 @@
           <t>factory</t>
         </is>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/factory</t>
         </is>
@@ -3988,7 +2779,7 @@
           <t>fampay</t>
         </is>
       </c>
-      <c r="B51" s="10" t="inlineStr">
+      <c r="B51" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/fampay</t>
         </is>
@@ -4016,7 +2807,7 @@
           <t>figma</t>
         </is>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B52" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/figma</t>
         </is>
@@ -4044,7 +2835,7 @@
           <t>fireworks</t>
         </is>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B53" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/fireworks</t>
         </is>
@@ -4072,7 +2863,7 @@
           <t>Freshworks</t>
         </is>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>https://careers.smartrecruiters.com/Freshworks</t>
         </is>
@@ -4100,7 +2891,7 @@
           <t>gamma</t>
         </is>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/gamma</t>
         </is>
@@ -4128,7 +2919,7 @@
           <t>gartner</t>
         </is>
       </c>
-      <c r="B56" s="10" t="inlineStr">
+      <c r="B56" s="11" t="inlineStr">
         <is>
           <t>https://gartner.wd5.myworkdayjobs.com/EXT</t>
         </is>
@@ -4156,7 +2947,7 @@
           <t>gitlab</t>
         </is>
       </c>
-      <c r="B57" s="10" t="inlineStr">
+      <c r="B57" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gitlab</t>
         </is>
@@ -4170,7 +2961,7 @@
         <v>232</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -4184,7 +2975,7 @@
           <t>glance</t>
         </is>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B58" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/glance</t>
         </is>
@@ -4212,7 +3003,7 @@
           <t>gradientai</t>
         </is>
       </c>
-      <c r="B59" s="10" t="inlineStr">
+      <c r="B59" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gradientai</t>
         </is>
@@ -4240,7 +3031,7 @@
           <t>groww</t>
         </is>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B60" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/groww</t>
         </is>
@@ -4268,7 +3059,7 @@
           <t>gusto</t>
         </is>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/gusto</t>
         </is>
@@ -4296,7 +3087,7 @@
           <t>harvey</t>
         </is>
       </c>
-      <c r="B62" s="10" t="inlineStr">
+      <c r="B62" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/harvey</t>
         </is>
@@ -4324,7 +3115,7 @@
           <t>hevodata</t>
         </is>
       </c>
-      <c r="B63" s="10" t="inlineStr">
+      <c r="B63" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/hevodata</t>
         </is>
@@ -4352,7 +3143,7 @@
           <t>highradius</t>
         </is>
       </c>
-      <c r="B64" s="10" t="inlineStr">
+      <c r="B64" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/highradius</t>
         </is>
@@ -4380,7 +3171,7 @@
           <t>hightouch</t>
         </is>
       </c>
-      <c r="B65" s="10" t="inlineStr">
+      <c r="B65" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/hightouch</t>
         </is>
@@ -4408,7 +3199,7 @@
           <t>hp</t>
         </is>
       </c>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="B66" s="11" t="inlineStr">
         <is>
           <t>https://hp.wd5.myworkdayjobs.com/ExternalCareerSite</t>
         </is>
@@ -4436,7 +3227,7 @@
           <t>ideogram</t>
         </is>
       </c>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="B67" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/ideogram</t>
         </is>
@@ -4464,7 +3255,7 @@
           <t>inmobi</t>
         </is>
       </c>
-      <c r="B68" s="10" t="inlineStr">
+      <c r="B68" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/inmobi</t>
         </is>
@@ -4492,7 +3283,7 @@
           <t>inngest</t>
         </is>
       </c>
-      <c r="B69" s="10" t="inlineStr">
+      <c r="B69" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/inngest</t>
         </is>
@@ -4520,7 +3311,7 @@
           <t>instacart</t>
         </is>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B70" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/instacart</t>
         </is>
@@ -4548,7 +3339,7 @@
           <t>intel</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B71" s="11" t="inlineStr">
         <is>
           <t>https://intel.wd1.myworkdayjobs.com/External</t>
         </is>
@@ -4576,7 +3367,7 @@
           <t>krea</t>
         </is>
       </c>
-      <c r="B72" s="10" t="inlineStr">
+      <c r="B72" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/krea</t>
         </is>
@@ -4604,7 +3395,7 @@
           <t>langchain</t>
         </is>
       </c>
-      <c r="B73" s="10" t="inlineStr">
+      <c r="B73" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/langchain</t>
         </is>
@@ -4632,7 +3423,7 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="B74" s="10" t="inlineStr">
+      <c r="B74" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/linear</t>
         </is>
@@ -4660,7 +3451,7 @@
           <t>llamaindex</t>
         </is>
       </c>
-      <c r="B75" s="10" t="inlineStr">
+      <c r="B75" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/llamaindex</t>
         </is>
@@ -4688,7 +3479,7 @@
           <t>lovable</t>
         </is>
       </c>
-      <c r="B76" s="10" t="inlineStr">
+      <c r="B76" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/lovable</t>
         </is>
@@ -4716,7 +3507,7 @@
           <t>lowes</t>
         </is>
       </c>
-      <c r="B77" s="10" t="inlineStr">
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>https://lowes.wd5.myworkdayjobs.com/LWS_External_CS</t>
         </is>
@@ -4744,7 +3535,7 @@
           <t>lyft</t>
         </is>
       </c>
-      <c r="B78" s="10" t="inlineStr">
+      <c r="B78" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/lyft</t>
         </is>
@@ -4772,7 +3563,7 @@
           <t>mastercard</t>
         </is>
       </c>
-      <c r="B79" s="10" t="inlineStr">
+      <c r="B79" s="11" t="inlineStr">
         <is>
           <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers</t>
         </is>
@@ -4786,7 +3577,7 @@
         <v>63</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4800,7 +3591,7 @@
           <t>meesho</t>
         </is>
       </c>
-      <c r="B80" s="10" t="inlineStr">
+      <c r="B80" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/meesho</t>
         </is>
@@ -4828,7 +3619,7 @@
           <t>microsoft</t>
         </is>
       </c>
-      <c r="B81" s="10" t="inlineStr">
+      <c r="B81" s="11" t="inlineStr">
         <is>
           <t>https://apply.careers.microsoft.com/careers?query=machine+learning&amp;location=India</t>
         </is>
@@ -4839,7 +3630,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E81" t="n">
         <v>0</v>
@@ -4856,7 +3647,7 @@
           <t>mindtickle</t>
         </is>
       </c>
-      <c r="B82" s="10" t="inlineStr">
+      <c r="B82" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/mindtickle</t>
         </is>
@@ -4884,7 +3675,7 @@
           <t>modal</t>
         </is>
       </c>
-      <c r="B83" s="10" t="inlineStr">
+      <c r="B83" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/modal</t>
         </is>
@@ -4912,7 +3703,7 @@
           <t>mongodb</t>
         </is>
       </c>
-      <c r="B84" s="10" t="inlineStr">
+      <c r="B84" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/mongodb</t>
         </is>
@@ -4940,7 +3731,7 @@
           <t>n8n</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B85" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/n8n</t>
         </is>
@@ -4968,7 +3759,7 @@
           <t>neon</t>
         </is>
       </c>
-      <c r="B86" s="10" t="inlineStr">
+      <c r="B86" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/neon</t>
         </is>
@@ -4996,7 +3787,7 @@
           <t>newrelic</t>
         </is>
       </c>
-      <c r="B87" s="10" t="inlineStr">
+      <c r="B87" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/newrelic</t>
         </is>
@@ -5024,7 +3815,7 @@
           <t>notion</t>
         </is>
       </c>
-      <c r="B88" s="10" t="inlineStr">
+      <c r="B88" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/notion</t>
         </is>
@@ -5052,7 +3843,7 @@
           <t>nvidia</t>
         </is>
       </c>
-      <c r="B89" s="10" t="inlineStr">
+      <c r="B89" s="11" t="inlineStr">
         <is>
           <t>https://nvidia.wd5.myworkdayjobs.com/NVIDIAExternalCareerSite</t>
         </is>
@@ -5080,7 +3871,7 @@
           <t>observeai</t>
         </is>
       </c>
-      <c r="B90" s="10" t="inlineStr">
+      <c r="B90" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/observeai</t>
         </is>
@@ -5108,7 +3899,7 @@
           <t>okta</t>
         </is>
       </c>
-      <c r="B91" s="10" t="inlineStr">
+      <c r="B91" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/okta</t>
         </is>
@@ -5136,7 +3927,7 @@
           <t>openai</t>
         </is>
       </c>
-      <c r="B92" s="10" t="inlineStr">
+      <c r="B92" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/openai</t>
         </is>
@@ -5150,7 +3941,7 @@
         <v>813</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -5164,7 +3955,7 @@
           <t>opusclip</t>
         </is>
       </c>
-      <c r="B93" s="10" t="inlineStr">
+      <c r="B93" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/opusclip</t>
         </is>
@@ -5192,7 +3983,7 @@
           <t>outreach</t>
         </is>
       </c>
-      <c r="B94" s="10" t="inlineStr">
+      <c r="B94" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/outreach</t>
         </is>
@@ -5220,7 +4011,7 @@
           <t>palantir</t>
         </is>
       </c>
-      <c r="B95" s="10" t="inlineStr">
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/palantir</t>
         </is>
@@ -5248,7 +4039,7 @@
           <t>paypal</t>
         </is>
       </c>
-      <c r="B96" s="10" t="inlineStr">
+      <c r="B96" s="11" t="inlineStr">
         <is>
           <t>https://paypal.wd1.myworkdayjobs.com/jobs</t>
         </is>
@@ -5276,7 +4067,7 @@
           <t>paytm</t>
         </is>
       </c>
-      <c r="B97" s="10" t="inlineStr">
+      <c r="B97" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/paytm</t>
         </is>
@@ -5304,7 +4095,7 @@
           <t>perplexity</t>
         </is>
       </c>
-      <c r="B98" s="10" t="inlineStr">
+      <c r="B98" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/perplexity</t>
         </is>
@@ -5332,7 +4123,7 @@
           <t>persona</t>
         </is>
       </c>
-      <c r="B99" s="10" t="inlineStr">
+      <c r="B99" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/persona</t>
         </is>
@@ -5360,7 +4151,7 @@
           <t>philips</t>
         </is>
       </c>
-      <c r="B100" s="10" t="inlineStr">
+      <c r="B100" s="11" t="inlineStr">
         <is>
           <t>https://philips.wd3.myworkdayjobs.com/jobs-and-careers</t>
         </is>
@@ -5374,7 +4165,7 @@
         <v>27</v>
       </c>
       <c r="E100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -5388,7 +4179,7 @@
           <t>pika</t>
         </is>
       </c>
-      <c r="B101" s="10" t="inlineStr">
+      <c r="B101" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/pika</t>
         </is>
@@ -5416,7 +4207,7 @@
           <t>pinecone</t>
         </is>
       </c>
-      <c r="B102" s="10" t="inlineStr">
+      <c r="B102" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/pinecone</t>
         </is>
@@ -5444,7 +4235,7 @@
           <t>pinterest</t>
         </is>
       </c>
-      <c r="B103" s="10" t="inlineStr">
+      <c r="B103" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/pinterest</t>
         </is>
@@ -5472,7 +4263,7 @@
           <t>plaid</t>
         </is>
       </c>
-      <c r="B104" s="10" t="inlineStr">
+      <c r="B104" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/plaid</t>
         </is>
@@ -5500,7 +4291,7 @@
           <t>pocketfm</t>
         </is>
       </c>
-      <c r="B105" s="10" t="inlineStr">
+      <c r="B105" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/pocketfm</t>
         </is>
@@ -5528,7 +4319,7 @@
           <t>poolside</t>
         </is>
       </c>
-      <c r="B106" s="10" t="inlineStr">
+      <c r="B106" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/poolside</t>
         </is>
@@ -5556,7 +4347,7 @@
           <t>porter</t>
         </is>
       </c>
-      <c r="B107" s="10" t="inlineStr">
+      <c r="B107" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/porter</t>
         </is>
@@ -5584,7 +4375,7 @@
           <t>posthog</t>
         </is>
       </c>
-      <c r="B108" s="10" t="inlineStr">
+      <c r="B108" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/posthog</t>
         </is>
@@ -5612,7 +4403,7 @@
           <t>prefect</t>
         </is>
       </c>
-      <c r="B109" s="10" t="inlineStr">
+      <c r="B109" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/prefect</t>
         </is>
@@ -5640,7 +4431,7 @@
           <t>pwc</t>
         </is>
       </c>
-      <c r="B110" s="10" t="inlineStr">
+      <c r="B110" s="11" t="inlineStr">
         <is>
           <t>https://pwc.wd3.myworkdayjobs.com/Global_Experienced_Careers</t>
         </is>
@@ -5668,7 +4459,7 @@
           <t>ramp</t>
         </is>
       </c>
-      <c r="B111" s="10" t="inlineStr">
+      <c r="B111" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/ramp</t>
         </is>
@@ -5696,7 +4487,7 @@
           <t>razorpaysoftwareprivatelimited</t>
         </is>
       </c>
-      <c r="B112" s="10" t="inlineStr">
+      <c r="B112" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/razorpaysoftwareprivatelimited</t>
         </is>
@@ -5724,7 +4515,7 @@
           <t>reddit</t>
         </is>
       </c>
-      <c r="B113" s="10" t="inlineStr">
+      <c r="B113" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/reddit</t>
         </is>
@@ -5752,7 +4543,7 @@
           <t>relevanceai</t>
         </is>
       </c>
-      <c r="B114" s="10" t="inlineStr">
+      <c r="B114" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/relevanceai</t>
         </is>
@@ -5780,7 +4571,7 @@
           <t>replit</t>
         </is>
       </c>
-      <c r="B115" s="10" t="inlineStr">
+      <c r="B115" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/replit</t>
         </is>
@@ -5808,7 +4599,7 @@
           <t>resend</t>
         </is>
       </c>
-      <c r="B116" s="10" t="inlineStr">
+      <c r="B116" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/resend</t>
         </is>
@@ -5836,7 +4627,7 @@
           <t>robinhood</t>
         </is>
       </c>
-      <c r="B117" s="10" t="inlineStr">
+      <c r="B117" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/robinhood</t>
         </is>
@@ -5864,7 +4655,7 @@
           <t>roblox</t>
         </is>
       </c>
-      <c r="B118" s="10" t="inlineStr">
+      <c r="B118" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/roblox</t>
         </is>
@@ -5892,7 +4683,7 @@
           <t>rubrik</t>
         </is>
       </c>
-      <c r="B119" s="10" t="inlineStr">
+      <c r="B119" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/rubrik</t>
         </is>
@@ -5920,7 +4711,7 @@
           <t>runway</t>
         </is>
       </c>
-      <c r="B120" s="10" t="inlineStr">
+      <c r="B120" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/runway</t>
         </is>
@@ -5948,7 +4739,7 @@
           <t>salesforce</t>
         </is>
       </c>
-      <c r="B121" s="10" t="inlineStr">
+      <c r="B121" s="11" t="inlineStr">
         <is>
           <t>https://salesforce.wd12.myworkdayjobs.com/External_Career_Site</t>
         </is>
@@ -5959,7 +4750,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E121" t="n">
         <v>0</v>
@@ -5976,7 +4767,7 @@
           <t>samsara</t>
         </is>
       </c>
-      <c r="B122" s="10" t="inlineStr">
+      <c r="B122" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/samsara</t>
         </is>
@@ -5987,7 +4778,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E122" t="n">
         <v>0</v>
@@ -6004,7 +4795,7 @@
           <t>sardine</t>
         </is>
       </c>
-      <c r="B123" s="10" t="inlineStr">
+      <c r="B123" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/sardine</t>
         </is>
@@ -6032,7 +4823,7 @@
           <t>sarvam</t>
         </is>
       </c>
-      <c r="B124" s="10" t="inlineStr">
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/sarvam</t>
         </is>
@@ -6046,7 +4837,7 @@
         <v>42</v>
       </c>
       <c r="E124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
@@ -6060,7 +4851,7 @@
           <t>scaleai</t>
         </is>
       </c>
-      <c r="B125" s="10" t="inlineStr">
+      <c r="B125" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/scaleai</t>
         </is>
@@ -6088,7 +4879,7 @@
           <t>ServiceNow</t>
         </is>
       </c>
-      <c r="B126" s="10" t="inlineStr">
+      <c r="B126" s="11" t="inlineStr">
         <is>
           <t>https://careers.smartrecruiters.com/ServiceNow</t>
         </is>
@@ -6116,7 +4907,7 @@
           <t>sierra</t>
         </is>
       </c>
-      <c r="B127" s="10" t="inlineStr">
+      <c r="B127" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/sierra</t>
         </is>
@@ -6144,7 +4935,7 @@
           <t>sigmoid</t>
         </is>
       </c>
-      <c r="B128" s="10" t="inlineStr">
+      <c r="B128" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/sigmoid</t>
         </is>
@@ -6172,7 +4963,7 @@
           <t>signoz</t>
         </is>
       </c>
-      <c r="B129" s="10" t="inlineStr">
+      <c r="B129" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/signoz</t>
         </is>
@@ -6200,7 +4991,7 @@
           <t>slice</t>
         </is>
       </c>
-      <c r="B130" s="10" t="inlineStr">
+      <c r="B130" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/slice</t>
         </is>
@@ -6228,7 +5019,7 @@
           <t>smallest</t>
         </is>
       </c>
-      <c r="B131" s="10" t="inlineStr">
+      <c r="B131" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/smallest</t>
         </is>
@@ -6256,7 +5047,7 @@
           <t>socure</t>
         </is>
       </c>
-      <c r="B132" s="10" t="inlineStr">
+      <c r="B132" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/socure</t>
         </is>
@@ -6284,7 +5075,7 @@
           <t>spotdraft</t>
         </is>
       </c>
-      <c r="B133" s="10" t="inlineStr">
+      <c r="B133" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/spotdraft</t>
         </is>
@@ -6312,7 +5103,7 @@
           <t>stripe</t>
         </is>
       </c>
-      <c r="B134" s="10" t="inlineStr">
+      <c r="B134" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/stripe</t>
         </is>
@@ -6340,7 +5131,7 @@
           <t>suno</t>
         </is>
       </c>
-      <c r="B135" s="10" t="inlineStr">
+      <c r="B135" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/suno</t>
         </is>
@@ -6368,7 +5159,7 @@
           <t>supabase</t>
         </is>
       </c>
-      <c r="B136" s="10" t="inlineStr">
+      <c r="B136" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/supabase</t>
         </is>
@@ -6396,7 +5187,7 @@
           <t>Swiggy</t>
         </is>
       </c>
-      <c r="B137" s="10" t="inlineStr">
+      <c r="B137" s="11" t="inlineStr">
         <is>
           <t>https://careers.smartrecruiters.com/Swiggy</t>
         </is>
@@ -6424,7 +5215,7 @@
           <t>synthesia</t>
         </is>
       </c>
-      <c r="B138" s="10" t="inlineStr">
+      <c r="B138" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/synthesia</t>
         </is>
@@ -6452,7 +5243,7 @@
           <t>tala</t>
         </is>
       </c>
-      <c r="B139" s="10" t="inlineStr">
+      <c r="B139" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/tala</t>
         </is>
@@ -6480,7 +5271,7 @@
           <t>target</t>
         </is>
       </c>
-      <c r="B140" s="10" t="inlineStr">
+      <c r="B140" s="11" t="inlineStr">
         <is>
           <t>https://target.wd5.myworkdayjobs.com/targetcareers</t>
         </is>
@@ -6508,7 +5299,7 @@
           <t>temporal</t>
         </is>
       </c>
-      <c r="B141" s="10" t="inlineStr">
+      <c r="B141" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/temporal</t>
         </is>
@@ -6536,7 +5327,7 @@
           <t>thomsonreuters</t>
         </is>
       </c>
-      <c r="B142" s="10" t="inlineStr">
+      <c r="B142" s="11" t="inlineStr">
         <is>
           <t>https://thomsonreuters.wd5.myworkdayjobs.com/External_Career_Site</t>
         </is>
@@ -6550,7 +5341,7 @@
         <v>24</v>
       </c>
       <c r="E142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -6564,7 +5355,7 @@
           <t>thoughtworks</t>
         </is>
       </c>
-      <c r="B143" s="10" t="inlineStr">
+      <c r="B143" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/thoughtworks</t>
         </is>
@@ -6592,7 +5383,7 @@
           <t>thoughtworks</t>
         </is>
       </c>
-      <c r="B144" s="10" t="inlineStr">
+      <c r="B144" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/thoughtworks</t>
         </is>
@@ -6620,7 +5411,7 @@
           <t>togetherai</t>
         </is>
       </c>
-      <c r="B145" s="10" t="inlineStr">
+      <c r="B145" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/togetherai</t>
         </is>
@@ -6648,7 +5439,7 @@
           <t>truefoundry</t>
         </is>
       </c>
-      <c r="B146" s="10" t="inlineStr">
+      <c r="B146" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/truefoundry</t>
         </is>
@@ -6676,7 +5467,7 @@
           <t>twilio</t>
         </is>
       </c>
-      <c r="B147" s="10" t="inlineStr">
+      <c r="B147" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/twilio</t>
         </is>
@@ -6704,7 +5495,7 @@
           <t>vercel</t>
         </is>
       </c>
-      <c r="B148" s="10" t="inlineStr">
+      <c r="B148" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/vercel</t>
         </is>
@@ -6732,7 +5523,7 @@
           <t>verkada</t>
         </is>
       </c>
-      <c r="B149" s="10" t="inlineStr">
+      <c r="B149" s="11" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/verkada</t>
         </is>
@@ -6760,7 +5551,7 @@
           <t>visa</t>
         </is>
       </c>
-      <c r="B150" s="10" t="inlineStr">
+      <c r="B150" s="11" t="inlineStr">
         <is>
           <t>https://visa.wd5.myworkdayjobs.com/Visa</t>
         </is>
@@ -6788,7 +5579,7 @@
           <t>warnerbros</t>
         </is>
       </c>
-      <c r="B151" s="10" t="inlineStr">
+      <c r="B151" s="11" t="inlineStr">
         <is>
           <t>https://warnerbros.wd5.myworkdayjobs.com/global</t>
         </is>
@@ -6802,7 +5593,7 @@
         <v>27</v>
       </c>
       <c r="E151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
@@ -6816,7 +5607,7 @@
           <t>warp</t>
         </is>
       </c>
-      <c r="B152" s="10" t="inlineStr">
+      <c r="B152" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/warp</t>
         </is>
@@ -6844,7 +5635,7 @@
           <t>weaviate</t>
         </is>
       </c>
-      <c r="B153" s="10" t="inlineStr">
+      <c r="B153" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/weaviate</t>
         </is>
@@ -6872,7 +5663,7 @@
           <t>workday</t>
         </is>
       </c>
-      <c r="B154" s="10" t="inlineStr">
+      <c r="B154" s="11" t="inlineStr">
         <is>
           <t>https://workday.wd5.myworkdayjobs.com/Workday</t>
         </is>
@@ -6900,7 +5691,7 @@
           <t>writer</t>
         </is>
       </c>
-      <c r="B155" s="10" t="inlineStr">
+      <c r="B155" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/writer</t>
         </is>
@@ -6928,7 +5719,7 @@
           <t>zapier</t>
         </is>
       </c>
-      <c r="B156" s="10" t="inlineStr">
+      <c r="B156" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/zapier</t>
         </is>
@@ -6956,7 +5747,7 @@
           <t>zed</t>
         </is>
       </c>
-      <c r="B157" s="10" t="inlineStr">
+      <c r="B157" s="11" t="inlineStr">
         <is>
           <t>https://jobs.ashbyhq.com/zed</t>
         </is>
@@ -6984,7 +5775,7 @@
           <t>zeta</t>
         </is>
       </c>
-      <c r="B158" s="10" t="inlineStr">
+      <c r="B158" s="11" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/zeta</t>
         </is>
@@ -7176,118 +5967,94 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
-        <is>
-          <t>Harpreet Singh Chhabra – AI Engineer &amp; Tech Lead (GenAI, Agentic AI, RAG, LLM Evaluation)</t>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Harpreet Singh Chhabra – AI Engineer &amp; Tech Lead (Agentic AI, LLM apps, RAG, LLM evaluation)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Search date</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>29 September 2026</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Target roles</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>AI Engineer, GenAI/LLM Engineer, Agentic AI / AI Agent Engineer, Applied AI Engineer, Forward Deployed Engineer, AI Solutions/Platform Engineer. Data Scientist / ML / Applied Scientist roles only when clearly LLM/agent work.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Locations</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>India (any city) or Remote roles open to India/Global. Remote roles restricted to US/EU/other countries were excluded.</t>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>India (any city) or remote roles open to India/Global.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Experience filter</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Posting's minimum required experience ≤ 2 years (or not stated and not a Senior/Staff/Lead/Manager title).</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Experience</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Posting's minimum required experience ≤ 2 years (or not stated and not Senior/Staff/Lead/Manager).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Only official company career pages / company-owned applicant tracking systems (Greenhouse, Lever, Ashby, Workday, SmartRecruiters, amazon.jobs, Microsoft Careers). No job aggregators (LinkedIn, Naukri, Indeed, etc.).</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Only official company career pages / company-hosted job boards (Greenhouse, Lever, Ashby, Workday, SmartRecruiters, amazon.jobs, Microsoft Careers). No aggregators.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Relevance</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Titles in AI/ML/GenAI/LLM/Agents/Applied Science/Forward-Deployed/Data Science, then each description read and scored against your resume (agents, tool calling, HITL, RAG, evals, semantic layers, Python/TypeScript).</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Link check</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Each run checks every link: HTTP 200 and posting still live on the company's careers system. Closed jobs are struck through, never deleted.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Link check</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Every apply link was fetched on 29-Sep-2026: HTTP 200, and the posting confirmed live via the company's careers API or the job title present on the page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Colour key</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Match score: green ≥85%, yellow 75–84%, orange &lt;75%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Excluded examples</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Roles needing 3+ yrs (e.g. Sarvam Agent Engineer, Notion FDE, Glance SDE II-ML, Microsoft Applied AI Scientist II), roles needing Master's/PhD, IIT-only, sales/MBA-type FDE roles.</t>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Match score: green ≥85%, yellow 75–84%, orange &lt;75%. Blue date = added on that run.</t>
         </is>
       </c>
     </row>

</xml_diff>